<commit_message>
Asignar nombres de integrantes en la distribución de la rúbrica CAT2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VG4xgdhKhBx7eX3sLMX2ij
</commit_message>
<xml_diff>
--- a/Rubrica_CAT2_EIN9967_distribucion_4_integrantes.xlsx
+++ b/Rubrica_CAT2_EIN9967_distribucion_4_integrantes.xlsx
@@ -44,25 +44,25 @@
     <t xml:space="preserve">Metodología: recolección y fuentes</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 1</t>
+    <t xml:space="preserve">Daniel</t>
   </si>
   <si>
     <t xml:space="preserve">Metodología: procesamiento + editor/a final</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 2</t>
+    <t xml:space="preserve">Claudia</t>
   </si>
   <si>
     <t xml:space="preserve">Resultados y conclusiones</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 3</t>
+    <t xml:space="preserve">César</t>
   </si>
   <si>
     <t xml:space="preserve">Análisis estratégico y planificación</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 4</t>
+    <t xml:space="preserve">Omar</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -887,16 +887,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1000,15 +1004,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1032,11 +1036,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1084,7 +1088,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1112,7 +1116,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1220,7 +1224,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1480,408 +1484,408 @@
   <dimension ref="B1:G28"/>
   <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="62"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="3"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="7" t="n">
+      <c r="E5" s="7"/>
+      <c r="F5" s="8" t="n">
         <f aca="false">SUMIF($E$12:$E$21,B5,$D$12:$D$21)</f>
         <v>25</v>
       </c>
-      <c r="G5" s="7"/>
+      <c r="G5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="10" t="n">
+      <c r="E6" s="7"/>
+      <c r="F6" s="11" t="n">
         <f aca="false">SUMIF($E$12:$E$21,B6,$D$12:$D$21)</f>
         <v>25</v>
       </c>
-      <c r="G6" s="10"/>
+      <c r="G6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="13" t="n">
+      <c r="E7" s="7"/>
+      <c r="F7" s="14" t="n">
         <f aca="false">SUMIF($E$12:$E$21,B7,$D$12:$D$21)</f>
         <v>25</v>
       </c>
-      <c r="G7" s="13"/>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="16" t="n">
+      <c r="E8" s="7"/>
+      <c r="F8" s="17" t="n">
         <f aca="false">SUMIF($E$12:$E$21,B8,$D$12:$D$21)</f>
         <v>25</v>
       </c>
-      <c r="G8" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C9" s="17" t="s">
+      <c r="G8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <f aca="false">SUM(F5:F8)</f>
         <v>100</v>
       </c>
-      <c r="G9" s="18"/>
+      <c r="G9" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I10</f>
         <v>15</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="23" t="str">
+      <c r="F12" s="24" t="str">
         <f aca="false">INDEX($D$5:$D$8,E12)</f>
-        <v>Integrante 1</v>
-      </c>
-      <c r="G12" s="20" t="s">
+        <v>Daniel</v>
+      </c>
+      <c r="G12" s="21" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I24</f>
         <v>5</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="23" t="str">
+      <c r="F13" s="24" t="str">
         <f aca="false">INDEX($D$5:$D$8,E13)</f>
-        <v>Integrante 1</v>
-      </c>
-      <c r="G13" s="20" t="s">
+        <v>Daniel</v>
+      </c>
+      <c r="G13" s="21" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I22</f>
         <v>5</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="23" t="str">
+      <c r="F14" s="24" t="str">
         <f aca="false">INDEX($D$5:$D$8,E14)</f>
-        <v>Integrante 1</v>
-      </c>
-      <c r="G14" s="20" t="s">
+        <v>Daniel</v>
+      </c>
+      <c r="G14" s="21" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I12</f>
         <v>15</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="24" t="str">
+      <c r="F15" s="25" t="str">
         <f aca="false">INDEX($D$5:$D$8,E15)</f>
-        <v>Integrante 2</v>
-      </c>
-      <c r="G15" s="20" t="s">
+        <v>Claudia</v>
+      </c>
+      <c r="G15" s="21" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I28</f>
         <v>10</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="24" t="str">
+      <c r="F16" s="25" t="str">
         <f aca="false">INDEX($D$5:$D$8,E16)</f>
-        <v>Integrante 2</v>
-      </c>
-      <c r="G16" s="20" t="s">
+        <v>Claudia</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I14</f>
         <v>15</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="25" t="str">
+      <c r="F17" s="26" t="str">
         <f aca="false">INDEX($D$5:$D$8,E17)</f>
-        <v>Integrante 3</v>
-      </c>
-      <c r="G17" s="20" t="s">
+        <v>César</v>
+      </c>
+      <c r="G17" s="21" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="19" t="n">
+      <c r="B18" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="21" t="n">
+      <c r="D18" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I20</f>
         <v>10</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="25" t="str">
+      <c r="F18" s="26" t="str">
         <f aca="false">INDEX($D$5:$D$8,E18)</f>
-        <v>Integrante 3</v>
-      </c>
-      <c r="G18" s="20" t="s">
+        <v>César</v>
+      </c>
+      <c r="G18" s="21" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="19" t="n">
+      <c r="B19" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="21" t="n">
+      <c r="D19" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I16</f>
         <v>10</v>
       </c>
-      <c r="E19" s="22" t="n">
+      <c r="E19" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="26" t="str">
+      <c r="F19" s="27" t="str">
         <f aca="false">INDEX($D$5:$D$8,E19)</f>
-        <v>Integrante 4</v>
-      </c>
-      <c r="G19" s="20" t="s">
+        <v>Omar</v>
+      </c>
+      <c r="G19" s="21" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="19" t="n">
+      <c r="B20" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="21" t="n">
+      <c r="D20" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I18</f>
         <v>10</v>
       </c>
-      <c r="E20" s="22" t="n">
+      <c r="E20" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="26" t="str">
+      <c r="F20" s="27" t="str">
         <f aca="false">INDEX($D$5:$D$8,E20)</f>
-        <v>Integrante 4</v>
-      </c>
-      <c r="G20" s="20" t="s">
+        <v>Omar</v>
+      </c>
+      <c r="G20" s="21" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="22" t="n">
         <f aca="false">'Rubrica CAT_2'!I26</f>
         <v>5</v>
       </c>
-      <c r="E21" s="22" t="n">
+      <c r="E21" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="26" t="str">
+      <c r="F21" s="27" t="str">
         <f aca="false">INDEX($D$5:$D$8,E21)</f>
-        <v>Integrante 4</v>
-      </c>
-      <c r="G21" s="20" t="s">
+        <v>Omar</v>
+      </c>
+      <c r="G21" s="21" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="17" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C22" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D22" s="27" t="n">
+      <c r="D22" s="28" t="n">
         <f aca="false">SUM(D12:D21)</f>
         <v>100</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="28" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="29" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="29" t="s">
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="29" t="s">
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C27" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="29" t="s">
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C28" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -1925,600 +1929,600 @@
   <dimension ref="B1:J31"/>
   <sheetFormatPr defaultColWidth="18" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="2.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="19.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="20.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="19.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="30" width="40.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="9.18"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="30" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="2.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="32" width="19.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="32" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="19.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="31" width="40.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="9.18"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="31" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D1" s="32" t="s">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="G4" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="36"/>
+      <c r="H4" s="37"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D5" s="34"/>
-      <c r="E5" s="37" t="s">
+      <c r="D5" s="35"/>
+      <c r="E5" s="38" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="40"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="42" t="s">
+      <c r="B9" s="41"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="43" t="s">
+      <c r="E9" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="F9" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="44" t="s">
+      <c r="G9" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="44" t="s">
+      <c r="H9" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="45" t="s">
+      <c r="I9" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="45" t="s">
+      <c r="J9" s="46" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="47" t="s">
+      <c r="D10" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="48" t="s">
+      <c r="E10" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="F10" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="48" t="s">
+      <c r="G10" s="49" t="s">
         <v>61</v>
       </c>
-      <c r="H10" s="48" t="s">
+      <c r="H10" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="49" t="n">
+      <c r="I10" s="50" t="n">
         <v>15</v>
       </c>
-      <c r="J10" s="50" t="str">
+      <c r="J10" s="51" t="str">
         <f aca="false">'Distribución 4 integrantes'!F12</f>
-        <v>Integrante 1</v>
+        <v>Daniel</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="51" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="52" t="s">
+      <c r="E11" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="52" t="s">
+      <c r="F11" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="52" t="s">
+      <c r="G11" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="H11" s="53" t="s">
+      <c r="H11" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="I11" s="49"/>
-      <c r="J11" s="50"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="51"/>
     </row>
     <row r="12" customFormat="false" ht="130.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="54" t="s">
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="55" t="s">
+      <c r="F12" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="G12" s="55" t="s">
+      <c r="G12" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="H12" s="55" t="s">
+      <c r="H12" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="I12" s="56" t="n">
+      <c r="I12" s="57" t="n">
         <v>15</v>
       </c>
-      <c r="J12" s="57" t="str">
+      <c r="J12" s="58" t="str">
         <f aca="false">'Distribución 4 integrantes'!F15</f>
-        <v>Integrante 2</v>
+        <v>Claudia</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="51" t="s">
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="52" t="s">
+      <c r="E13" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="F13" s="52" t="s">
+      <c r="F13" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="52" t="s">
+      <c r="G13" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="H13" s="53" t="s">
+      <c r="H13" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="I13" s="56"/>
-      <c r="J13" s="57"/>
+      <c r="I13" s="57"/>
+      <c r="J13" s="58"/>
     </row>
     <row r="14" customFormat="false" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="47" t="s">
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="58" t="s">
+      <c r="E14" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="59" t="s">
+      <c r="F14" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="58" t="s">
+      <c r="G14" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="H14" s="58" t="s">
+      <c r="H14" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="49" t="n">
+      <c r="I14" s="50" t="n">
         <v>15</v>
       </c>
-      <c r="J14" s="60" t="str">
+      <c r="J14" s="61" t="str">
         <f aca="false">'Distribución 4 integrantes'!F17</f>
-        <v>Integrante 3</v>
+        <v>César</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="51" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="52" t="s">
+      <c r="E15" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="52" t="s">
+      <c r="F15" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="G15" s="52" t="s">
+      <c r="G15" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="H15" s="53" t="s">
+      <c r="H15" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="I15" s="49"/>
-      <c r="J15" s="60"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="61"/>
     </row>
     <row r="16" customFormat="false" ht="198" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="46"/>
-      <c r="C16" s="61" t="s">
+      <c r="B16" s="47"/>
+      <c r="C16" s="62" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="54" t="s">
+      <c r="D16" s="55" t="s">
         <v>79</v>
       </c>
-      <c r="E16" s="62" t="s">
+      <c r="E16" s="63" t="s">
         <v>80</v>
       </c>
-      <c r="F16" s="62" t="s">
+      <c r="F16" s="63" t="s">
         <v>81</v>
       </c>
-      <c r="G16" s="62" t="s">
+      <c r="G16" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="62" t="s">
+      <c r="H16" s="63" t="s">
         <v>83</v>
       </c>
-      <c r="I16" s="56" t="n">
+      <c r="I16" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="J16" s="63" t="str">
+      <c r="J16" s="64" t="str">
         <f aca="false">'Distribución 4 integrantes'!F19</f>
-        <v>Integrante 4</v>
+        <v>Omar</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="46"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="51" t="s">
+      <c r="B17" s="47"/>
+      <c r="C17" s="62"/>
+      <c r="D17" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="52" t="s">
+      <c r="E17" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F17" s="52" t="s">
+      <c r="F17" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="G17" s="52" t="s">
+      <c r="G17" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="56"/>
-      <c r="J17" s="63"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="64"/>
     </row>
     <row r="18" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="46"/>
-      <c r="C18" s="64" t="s">
+      <c r="B18" s="47"/>
+      <c r="C18" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="D18" s="47" t="s">
+      <c r="D18" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="58" t="s">
+      <c r="E18" s="59" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="65" t="s">
+      <c r="F18" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="G18" s="66" t="s">
+      <c r="G18" s="67" t="s">
         <v>91</v>
       </c>
-      <c r="H18" s="67" t="s">
+      <c r="H18" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="I18" s="49" t="n">
+      <c r="I18" s="50" t="n">
         <v>10</v>
       </c>
-      <c r="J18" s="63" t="str">
+      <c r="J18" s="64" t="str">
         <f aca="false">'Distribución 4 integrantes'!F20</f>
-        <v>Integrante 4</v>
+        <v>Omar</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="46"/>
-      <c r="C19" s="64"/>
-      <c r="D19" s="51" t="s">
+      <c r="B19" s="47"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="52" t="s">
+      <c r="E19" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F19" s="52" t="s">
+      <c r="F19" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="G19" s="52" t="s">
+      <c r="G19" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="53" t="s">
+      <c r="H19" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="I19" s="49"/>
-      <c r="J19" s="63"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="64"/>
     </row>
     <row r="20" customFormat="false" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="68" t="s">
+      <c r="B20" s="69" t="s">
         <v>93</v>
       </c>
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="62" t="s">
         <v>94</v>
       </c>
-      <c r="D20" s="54" t="s">
+      <c r="D20" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="69" t="s">
+      <c r="E20" s="70" t="s">
         <v>95</v>
       </c>
-      <c r="F20" s="70" t="s">
+      <c r="F20" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="G20" s="70" t="s">
+      <c r="G20" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="H20" s="71" t="s">
+      <c r="H20" s="72" t="s">
         <v>98</v>
       </c>
-      <c r="I20" s="56" t="n">
+      <c r="I20" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="J20" s="60" t="str">
+      <c r="J20" s="61" t="str">
         <f aca="false">'Distribución 4 integrantes'!F18</f>
-        <v>Integrante 3</v>
+        <v>César</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="68"/>
-      <c r="C21" s="68"/>
-      <c r="D21" s="51" t="s">
+      <c r="B21" s="69"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="52" t="s">
+      <c r="E21" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F21" s="52" t="s">
+      <c r="F21" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="G21" s="52" t="s">
+      <c r="G21" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="53" t="s">
+      <c r="H21" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="I21" s="56"/>
-      <c r="J21" s="60"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="61"/>
     </row>
     <row r="22" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="47" t="s">
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="58" t="s">
+      <c r="E22" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="F22" s="72" t="s">
+      <c r="F22" s="73" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="66" t="s">
+      <c r="G22" s="67" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="67" t="s">
+      <c r="H22" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="I22" s="49" t="n">
+      <c r="I22" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="J22" s="50" t="str">
+      <c r="J22" s="51" t="str">
         <f aca="false">'Distribución 4 integrantes'!F14</f>
-        <v>Integrante 1</v>
+        <v>Daniel</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="68"/>
-      <c r="C23" s="61"/>
-      <c r="D23" s="51" t="s">
+      <c r="B23" s="69"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E23" s="52" t="s">
+      <c r="E23" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="F23" s="52" t="s">
+      <c r="F23" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="G23" s="52" t="s">
+      <c r="G23" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="53" t="s">
+      <c r="H23" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="I23" s="49"/>
-      <c r="J23" s="50"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="51"/>
     </row>
     <row r="24" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="61" t="s">
+      <c r="B24" s="62" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="73" t="s">
+      <c r="C24" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="D24" s="74" t="s">
+      <c r="D24" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="75" t="s">
+      <c r="E24" s="76" t="s">
         <v>108</v>
       </c>
-      <c r="F24" s="70" t="s">
+      <c r="F24" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="G24" s="70" t="s">
+      <c r="G24" s="71" t="s">
         <v>110</v>
       </c>
-      <c r="H24" s="71" t="s">
+      <c r="H24" s="72" t="s">
         <v>111</v>
       </c>
-      <c r="I24" s="56" t="n">
+      <c r="I24" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="J24" s="50" t="str">
+      <c r="J24" s="51" t="str">
         <f aca="false">'Distribución 4 integrantes'!F13</f>
-        <v>Integrante 1</v>
+        <v>Daniel</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="61"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="51" t="s">
+      <c r="B25" s="62"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E25" s="52" t="s">
+      <c r="E25" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="F25" s="52" t="s">
+      <c r="F25" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="G25" s="52" t="s">
+      <c r="G25" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="H25" s="53" t="s">
+      <c r="H25" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="I25" s="56"/>
-      <c r="J25" s="50"/>
+      <c r="I25" s="57"/>
+      <c r="J25" s="51"/>
     </row>
     <row r="26" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="C26" s="76" t="s">
+      <c r="C26" s="77" t="s">
         <v>112</v>
       </c>
-      <c r="D26" s="77" t="s">
+      <c r="D26" s="78" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="55" t="s">
+      <c r="E26" s="56" t="s">
         <v>113</v>
       </c>
-      <c r="F26" s="55" t="s">
+      <c r="F26" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="G26" s="78" t="s">
+      <c r="G26" s="79" t="s">
         <v>115</v>
       </c>
-      <c r="H26" s="78" t="s">
+      <c r="H26" s="79" t="s">
         <v>116</v>
       </c>
-      <c r="I26" s="56" t="n">
+      <c r="I26" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="63" t="str">
+      <c r="J26" s="64" t="str">
         <f aca="false">'Distribución 4 integrantes'!F21</f>
-        <v>Integrante 4</v>
+        <v>Omar</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="46"/>
-      <c r="C27" s="76"/>
-      <c r="D27" s="51" t="s">
+      <c r="B27" s="47"/>
+      <c r="C27" s="77"/>
+      <c r="D27" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="79" t="s">
+      <c r="E27" s="80" t="s">
         <v>103</v>
       </c>
-      <c r="F27" s="79" t="s">
+      <c r="F27" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="G27" s="79" t="s">
+      <c r="G27" s="80" t="s">
         <v>105</v>
       </c>
-      <c r="H27" s="80" t="s">
+      <c r="H27" s="81" t="s">
         <v>106</v>
       </c>
-      <c r="I27" s="56"/>
-      <c r="J27" s="63"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="64"/>
     </row>
     <row r="28" customFormat="false" ht="81" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="61" t="s">
+      <c r="B28" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="C28" s="61" t="s">
+      <c r="C28" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="81" t="s">
+      <c r="D28" s="82" t="s">
         <v>119</v>
       </c>
-      <c r="E28" s="55" t="s">
+      <c r="E28" s="56" t="s">
         <v>120</v>
       </c>
-      <c r="F28" s="55" t="s">
+      <c r="F28" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="G28" s="78" t="s">
+      <c r="G28" s="79" t="s">
         <v>122</v>
       </c>
-      <c r="H28" s="78" t="s">
+      <c r="H28" s="79" t="s">
         <v>123</v>
       </c>
-      <c r="I28" s="56" t="n">
+      <c r="I28" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="J28" s="57" t="str">
+      <c r="J28" s="58" t="str">
         <f aca="false">'Distribución 4 integrantes'!F16</f>
-        <v>Integrante 2</v>
+        <v>Claudia</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="61"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="82" t="s">
+      <c r="B29" s="62"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="52" t="s">
+      <c r="E29" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F29" s="52" t="s">
+      <c r="F29" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="52" t="s">
+      <c r="G29" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="H29" s="53" t="s">
+      <c r="H29" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="I29" s="56"/>
-      <c r="J29" s="57"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="58"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I30" s="83" t="n">
+      <c r="I30" s="84" t="n">
         <f aca="false">SUM(I10:I29)</f>
         <v>100</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D31" s="84"/>
+      <c r="D31" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="35">

</xml_diff>